<commit_message>
Updates sample batch payment links file
</commit_message>
<xml_diff>
--- a/public/files/sample_batch_payment_links.xlsx
+++ b/public/files/sample_batch_payment_links.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="18315"/>
   <workbookPr/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{76F9B298-3EC5-4DCC-8F36-03205DC11709}" xr6:coauthVersionLast="20" xr6:coauthVersionMax="20" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{AC73F1F5-4396-4A37-950C-C301489A8B28}" xr6:coauthVersionLast="20" xr6:coauthVersionMax="20" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="11">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
   <si>
     <t>Invoice Number</t>
   </si>
@@ -36,6 +36,9 @@
   </si>
   <si>
     <t>Expire By</t>
+  </si>
+  <si>
+    <t>Partial Payment</t>
   </si>
   <si>
     <t>#1</t>
@@ -400,7 +403,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G2"/>
+  <dimension ref="A1:H2"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="18.5703125" customWidth="1"/>
@@ -412,7 +415,7 @@
     <col min="7" max="7" width="14.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7">
+    <row r="1" spans="1:8">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -434,16 +437,19 @@
       <c r="G1" t="s">
         <v>6</v>
       </c>
+      <c r="H1" t="s">
+        <v>7</v>
+      </c>
     </row>
-    <row r="2" spans="1:7">
+    <row r="2" spans="1:8">
       <c r="A2" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B2" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D2">
         <v>9999988888</v>
@@ -452,7 +458,10 @@
         <v>100</v>
       </c>
       <c r="F2" t="s">
-        <v>10</v>
+        <v>11</v>
+      </c>
+      <c r="H2">
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>